<commit_message>
feat(forward): liquidar 117 pendencias historicas de agosto e setembro com dados oficiais
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-19.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-19.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sinais_Aprovados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -686,19 +686,19 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>vs</t>
+          <t>0x1</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>🟢 GREEN</t>
         </is>
       </c>
       <c r="S3" t="n">
@@ -1105,19 +1105,19 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>vs</t>
+          <t>0x0</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>🟢 GREEN</t>
         </is>
       </c>
       <c r="S8" t="n">

</xml_diff>